<commit_message>
feat(geography): nest name as {th, en} for schema consistency (v3.1)
v3.0.0 left geography.name as a flat string while every other entity moved
to nested {th, en}. This closes that last inconsistency.

- data/spec/geography.json: name type string -> object {th, en}
- data/raw/geographies.json: 6 regions given English names (adjective form:
  Northern, Central, Northeastern, Western, Eastern, Southern)
- 1_export_file_format.py: COLUMN_ORDER + DDL for geographies use
  name_th/name_en; flatten_row already handled nested name generically
- formats/{csv,json,sql,xlsx,xml}/geographies regenerated
- api/latest unchanged (geography is not an API entity; province.geography_id
  stays an int FK)
- Docs: CHANGELOG v3.1.0 entry, schema.md, diagram.md, README/README.en

No prefix field for geography (regions have no prefix concept; unlike
province which carries prefix:null).
</commit_message>
<xml_diff>
--- a/formats/xlsx/geographies.xlsx
+++ b/formats/xlsx/geographies.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,7 +424,12 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>name_th</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>name_en</t>
         </is>
       </c>
     </row>
@@ -437,6 +442,11 @@
           <t>ภาคเหนือ</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Northern</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -447,6 +457,11 @@
           <t>ภาคกลาง</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Central</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -457,6 +472,11 @@
           <t>ภาคตะวันออกเฉียงเหนือ</t>
         </is>
       </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Northeastern</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -467,6 +487,11 @@
           <t>ภาคตะวันตก</t>
         </is>
       </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Western</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -477,6 +502,11 @@
           <t>ภาคตะวันออก</t>
         </is>
       </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Eastern</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -485,6 +515,11 @@
       <c r="B7" t="inlineStr">
         <is>
           <t>ภาคใต้</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Southern</t>
         </is>
       </c>
     </row>

</xml_diff>